<commit_message>
-Double-checking -Edits to figures saved as additional copies (assessing PLA & SA separately)
</commit_message>
<xml_diff>
--- a/data/raw/4_LA_Corrections_DK.xlsx
+++ b/data/raw/4_LA_Corrections_DK.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Work\Masters\Minimum Conductance\Huw_min_cond (working ver)\Projected Leaf area versions\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/01424892_wf_uct_ac_za/Documents/Adam Data OneDrive/Adam Manuscripts/irlam/gmin_methodology_paper-main/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558DED8C-ED2B-43B2-894D-7A7B1884551B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{558DED8C-ED2B-43B2-894D-7A7B1884551B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3250D99-68FC-6749-A90F-68728A12724C}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{C416B5F1-D903-498C-983A-F0F8E0771570}"/>
+    <workbookView xWindow="37320" yWindow="600" windowWidth="33140" windowHeight="19820" xr2:uid="{C416B5F1-D903-498C-983A-F0F8E0771570}"/>
   </bookViews>
   <sheets>
     <sheet name="LeafArea_Corrections+Transforma" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1017,14 +1017,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDB93D7D-4FBB-46B3-B362-F786A39B04D3}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -1041,7 +1042,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1059,7 +1060,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1078,7 +1079,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1096,7 +1097,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1115,7 +1116,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1133,7 +1134,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1152,7 +1153,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1170,7 +1171,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1189,7 +1190,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -1207,7 +1208,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1225,7 +1226,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -1243,7 +1244,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1261,7 +1262,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -1279,17 +1280,17 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D19" t="s">
         <v>33</v>
       </c>

</xml_diff>